<commit_message>
feat(content): 补充 tasks/channels 的 Excel 模板与导入，校验渠道表
</commit_message>
<xml_diff>
--- a/content/balance.xlsx
+++ b/content/balance.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>key</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t>divinationBase</t>
+  </si>
+  <si>
+    <t>partyMax</t>
   </si>
   <si>
     <t>commonPrice</t>
@@ -444,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -560,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>800</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -568,6 +571,14 @@
         <v>15</v>
       </c>
       <c r="B15">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16">
         <v>2000</v>
       </c>
     </row>

</xml_diff>